<commit_message>
feat(v6.3.0): switch all recommendations to advisory tone
Replace commands and growth guarantees with suggestion language across PDF, UI, AI prompts, and extension badges. Add an advisory-tone pytest suite scoped to tests/ via pytest.ini.
</commit_message>
<xml_diff>
--- a/translations.xlsx
+++ b/translations.xlsx
@@ -922,17 +922,17 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>SEO için ne yapmalıyım?</t>
+          <t>SEO için ne yapabilirim?</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>What should I do for SEO?</t>
+          <t>What could I do for SEO?</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>¿Qué debo hacer para el SEO?</t>
+          <t>¿Qué podría hacer para el SEO?</t>
         </is>
       </c>
     </row>
@@ -1010,17 +1010,17 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Thumbnail nasıl olmalı?</t>
+          <t>Thumbnail nasıl olabilir?</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>How should the thumbnail be?</t>
+          <t>How could the thumbnail look?</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>¿Cómo debería ser la miniatura?</t>
+          <t>¿Cómo podría ser la miniatura?</t>
         </is>
       </c>
     </row>
@@ -3188,17 +3188,17 @@
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>Bu rakibin etiketlerini kopyalamak algoritmayı karıştırır. PDF Raporundaki etiket önerileri bu rakip için devre dışı bırakıldı.</t>
+          <t>Bu rakibin etiketlerini kopyalamak algoritmayı karıştırabilir. PDF Raporundaki etiket önerileri bu rakip için devre dışı bırakıldı.</t>
         </is>
       </c>
       <c r="C125" s="3" t="inlineStr">
         <is>
-          <t>Copying this competitor's tags will confuse the algorithm. Tag suggestions in the PDF Report have been disabled for this competitor.</t>
+          <t>Copying this competitor's tags could confuse the algorithm. Tag suggestions in the PDF Report have been disabled for this competitor.</t>
         </is>
       </c>
       <c r="D125" s="3" t="inlineStr">
         <is>
-          <t>Copiar las etiquetas de este competidor confundirá al algoritmo. Las sugerencias de etiquetas en el Informe PDF se han desactivado para este competidor.</t>
+          <t>Copiar las etiquetas de este competidor podría confundir al algoritmo. Las sugerencias de etiquetas en el Informe PDF se han desactivado para este competidor.</t>
         </is>
       </c>
     </row>
@@ -4068,17 +4068,17 @@
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>Şimdi şunları yap:</t>
+          <t>Bu durumda şunları deneyebilirsin:</t>
         </is>
       </c>
       <c r="C165" s="3" t="inlineStr">
         <is>
-          <t>Do these now:</t>
+          <t>In this situation you could try:</t>
         </is>
       </c>
       <c r="D165" s="3" t="inlineStr">
         <is>
-          <t>Haz esto ahora:</t>
+          <t>En esta situación podrías probar:</t>
         </is>
       </c>
     </row>
@@ -4286,17 +4286,17 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>VİRAL OLMA ŞANSINI KAYBEDİYORSUN!</t>
+          <t>VİRAL POTANSİYELİN RİSK ALTINDA OLABİLİR</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>YOU'RE LOSING YOUR VIRAL CHANCE!</t>
+          <t>YOUR VIRAL POTENTIAL MAY BE AT RISK</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>¡ESTÁS PERDIENDO TU OPORTUNIDAD VIRAL!</t>
+          <t>TU POTENCIAL VIRAL PODRÍA ESTAR EN RIESGO</t>
         </is>
       </c>
     </row>
@@ -4682,17 +4682,17 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Başlığındaki anahtar kelimeler etiketlerde neredeyse hiç geçmiyor. Algoritma videoyu yanlış kitleye gösterir.</t>
+          <t>Başlığındaki anahtar kelimeler etiketlerde neredeyse hiç geçmiyor. Bu durumda algoritma videoyu yanlış kitleye gösterebilir.</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Keywords in your title are barely present in your tags. The algorithm will show your video to the wrong audience.</t>
+          <t>Keywords in your title are barely present in your tags. In this case the algorithm may show your video to the wrong audience.</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Las palabras clave de tu título apenas aparecen en tus etiquetas. El algoritmo mostrará tu video a la audiencia equivocada.</t>
+          <t>Las palabras clave de tu título apenas aparecen en tus etiquetas. En ese caso el algoritmo podría mostrar tu video a la audiencia equivocada.</t>
         </is>
       </c>
     </row>
@@ -4726,17 +4726,17 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Açıklaman başlıkla alakasız kelimeler içeriyor. SEO puanın düşer.</t>
+          <t>Açıklaman başlıkla alakasız kelimeler içeriyor. Bu, SEO puanını düşürebilir.</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Your description contains words unrelated to the title. Your SEO score will drop.</t>
+          <t>Your description contains words unrelated to the title. This may lower your SEO score.</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Tu descripción contiene palabras no relacionadas con el título. Tu puntuación SEO bajará.</t>
+          <t>Tu descripción contiene palabras no relacionadas con el título. Esto podría bajar tu puntuación SEO.</t>
         </is>
       </c>
     </row>
@@ -4902,17 +4902,17 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Ne Yapmalısın?</t>
+          <t>Ne Yapabilirsin?</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>What Should You Do?</t>
+          <t>What Could You Do?</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>¿Qué Deberías Hacer?</t>
+          <t>¿Qué Podrías Hacer?</t>
         </is>
       </c>
     </row>
@@ -4924,17 +4924,17 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>• İnternetini kontrol et ve analizi tekrar başlat</t>
+          <t>• İnternetini kontrol edip analizi tekrar başlatabilirsin</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>• Check your internet and restart the analysis</t>
+          <t>• You could check your internet and restart the analysis</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>• Verifica tu internet y reinicia el análisis</t>
+          <t>• Podrías verificar tu internet y reiniciar el análisis</t>
         </is>
       </c>
     </row>
@@ -4946,17 +4946,17 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>• Ya da rakip video URL'sini elle girerek yeniden analiz yap</t>
+          <t>• Ya da rakip video URL'sini elle girerek yeniden analiz edebilirsin</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>• Or manually enter a competitor video URL and re-analyze</t>
+          <t>• Or you could manually enter a competitor video URL and re-analyze</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>• O ingresa manualmente una URL de video competidor y vuelve a analizar</t>
+          <t>• O podrías ingresar manualmente una URL de video competidor y volver a analizar</t>
         </is>
       </c>
     </row>
@@ -5012,17 +5012,17 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>* AI Notu: Bunlar 'Ölü Okyanus'tur. Buradan yeni izleyici gelmez, etiket kotanı israf edersin.</t>
+          <t>* AI Notu: Bunlar 'Ölü Okyanus' sayılır. Buradan yeni izleyici gelmesi zor olabilir ve etiket kotan boşa gidebilir.</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>* AI Note: These are 'Dead Oceans'. No new viewers will come from here, you're wasting your tag quota.</t>
+          <t>* AI Note: These count as 'Dead Oceans'. New viewers rarely come from here, and your tag quota may go to waste.</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>* Nota IA: Estos son 'Océanos Muertos'. No vendrán nuevos espectadores desde aquí, estás desperdiciando tu cuota de etiquetas.</t>
+          <t>* Nota IA: Estos se consideran 'Océanos Muertos'. Es difícil que lleguen nuevos espectadores desde aquí y tu cuota de etiquetas podría desaprovecharse.</t>
         </is>
       </c>
     </row>
@@ -5056,17 +5056,17 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>* AI Notu: Bu kelimeler başlığında veya açıklama konseptinde HİÇ geçmiyor! Yanlış kitlenin tıklayıp hemen çıkmasına sebep olur. Retention'ı öldürür! Derhal sil.</t>
+          <t>* AI Notu: Bu kelimeler başlığında veya açıklama konseptinde geçmiyor. Yanlış kitlenin tıklayıp hemen çıkmasına yol açabilir ve retention'ı düşürebilir. Bu etiketleri kaldırmayı düşünebilirsin.</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>* AI Note: These words don't appear in your title or description at all! They cause wrong audiences to click and leave immediately. Destroys retention! Delete immediately.</t>
+          <t>* AI Note: These words don't appear in your title or description concept. They may lead the wrong audience to click and leave immediately, which can lower your retention. You could consider removing them.</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>* Nota IA: ¡Estas palabras no aparecen en tu título o descripción! Causan que audiencias equivocadas hagan clic y se vayan inmediatamente. ¡Destruye la retención! Elimínalas inmediatamente.</t>
+          <t>* Nota IA: Estas palabras no aparecen en tu título ni en el concepto de tu descripción. Pueden hacer que la audiencia equivocada haga clic y se vaya enseguida, lo que puede reducir la retención. Podrías considerar eliminarlas.</t>
         </is>
       </c>
     </row>
@@ -5144,17 +5144,17 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>* AI Notu: Videonla gram alakası olmayan hashtagleri kullanmak kanalın otoritesine zarar verir!</t>
+          <t>* AI Notu: Videonla alakası olmayan hashtagler kanalının otoritesine zarar verebilir.</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>* AI Note: Using hashtags completely unrelated to your video damages your channel authority!</t>
+          <t>* AI Note: Using hashtags unrelated to your video may weaken your channel authority.</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>* Nota IA: ¡Usar hashtags completamente no relacionados con tu video daña la autoridad de tu canal!</t>
+          <t>* Nota IA: Usar hashtags no relacionados con tu video puede debilitar la autoridad de tu canal.</t>
         </is>
       </c>
     </row>
@@ -5188,17 +5188,17 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Açıklamaya hiç hashtag girmemişsin! (Öneri: Açıklamanın sonuna içeriğini anlatan en fazla 3 adet # ekle)</t>
+          <t>Açıklamaya hiç hashtag girilmemiş. (Öneri: Açıklamanın sonuna içeriğini anlatan en fazla 3 adet # ekleyebilirsin)</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>You haven't added any hashtags to the description! (Suggestion: Add up to 3 relevant hashtags at the end of your description)</t>
+          <t>No hashtags have been added to the description. (Suggestion: you could add up to 3 relevant hashtags at the end of your description)</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>¡No has añadido ningún hashtag a la descripción! (Sugerencia: Añade hasta 3 hashtags relevantes al final de tu descripción)</t>
+          <t>No se han añadido hashtags a la descripción. (Sugerencia: podrías añadir hasta 3 hashtags relevantes al final de tu descripción)</t>
         </is>
       </c>
     </row>
@@ -5606,17 +5606,17 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Rakip başlığında çok daha fazla detay vererek kitleyi meraklandırmayı başarmış. Başlıklarını uzatmalısın!</t>
+          <t>Rakip başlığında çok daha fazla detay vererek kitleyi meraklandırmayı başarmış. Başlıklarını biraz uzatmayı deneyebilirsin.</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>The competitor added much more detail to their title to intrigue the audience. You should make your titles longer!</t>
+          <t>The competitor added much more detail to their title to intrigue the audience. You could try making your titles a bit longer.</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>¡El competidor añadió mucho más detalle a su título para intrigar a la audiencia. Deberías hacer tus títulos más largos!</t>
+          <t>El competidor añadió mucho más detalle a su título para intrigar a la audiencia. Podrías probar a hacer tus títulos un poco más largos.</t>
         </is>
       </c>
     </row>
@@ -5672,17 +5672,17 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>⚠️ Konsept uyumsuzluğu var — aşağıdaki etiketleri kör kopyalamak yerine kendi içeriğine uyanları seç.</t>
+          <t>⚠️ Konsept uyumsuzluğu var — aşağıdaki etiketleri kör kopyalamak yerine kendi içeriğine uyanları seçebilirsin.</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>⚠️ Concept mismatch — instead of blindly copying, select only the tags that match your content.</t>
+          <t>⚠️ Concept mismatch — instead of blindly copying, you could pick only the tags that match your content.</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>⚠️ Desajuste de concepto — en lugar de copiar ciegamente, selecciona solo las etiquetas que coincidan con tu contenido.</t>
+          <t>⚠️ Desajuste de concepto — en lugar de copiar ciegamente, podrías elegir solo las etiquetas que coincidan con tu contenido.</t>
         </is>
       </c>
     </row>
@@ -5694,17 +5694,17 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>🎯 Videonla %100 Uyumlu Olanlar (KESİN EKLE)</t>
+          <t>🎯 Videonla %100 Uyumlu Olanlar (Ekleyebilirsin)</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>🎯 100% Compatible with Your Video (DEFINITELY ADD)</t>
+          <t>🎯 100% Compatible with Your Video (You Could Add These)</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>🎯 100% Compatible con Tu Video (AÑADE DEFINITIVAMENTE)</t>
+          <t>🎯 100% Compatible con Tu Video (Podrías Añadirlas)</t>
         </is>
       </c>
     </row>
@@ -5716,17 +5716,17 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>⚠️ İlham Havuzu (Seçerek Kullan)</t>
+          <t>⚠️ İlham Havuzu (Seçerek Kullanabilirsin)</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>⚠️ Inspiration Pool (Use Selectively)</t>
+          <t>⚠️ Inspiration Pool (You Could Use Selectively)</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>⚠️ Grupo de Inspiración (Usar Selectivamente)</t>
+          <t>⚠️ Grupo de Inspiración (Podrías Usarlas Selectivamente)</t>
         </is>
       </c>
     </row>
@@ -5738,17 +5738,17 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>⛔ KESİNLİKLE UZAK DUR (Zehirli Etiketler)</t>
+          <t>⛔ Uzak Durman Önerilir (Riskli Etiketler)</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>⛔ AVOID COMPLETELY (Toxic Tags)</t>
+          <t>⛔ Best Avoided (Risky Tags)</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>⛔ EVITAR COMPLETAMENTE (Etiquetas Tóxicas)</t>
+          <t>⛔ Mejor Evitarlas (Etiquetas Riesgosas)</t>
         </is>
       </c>
     </row>
@@ -5760,17 +5760,17 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>* AI Notu: Eklersen algoritma videonu yanlış kitleye gösterir ve izlenmen donar.</t>
+          <t>* AI Notu: Eklersen algoritma videonu yanlış kitleye gösterebilir ve izlenmen yavaşlayabilir.</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>* AI Note: Adding these will make the algorithm show your video to the wrong audience and freeze your views.</t>
+          <t>* AI Note: Adding these could make the algorithm show your video to the wrong audience and slow down your views.</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>* Nota IA: Añadir estas hará que el algoritmo muestre tu video a la audiencia equivocada y congele tus vistas.</t>
+          <t>* Nota IA: Añadirlas podría hacer que el algoritmo muestre tu video a la audiencia equivocada y ralentice tus vistas.</t>
         </is>
       </c>
     </row>
@@ -5782,17 +5782,17 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>#️⃣ Rakibinden Çalınabilecek Hashtagler</t>
+          <t>#️⃣ Rakibinden İlham Alabileceğin Hashtagler</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>#️⃣ Hashtags to Steal from Competitor</t>
+          <t>#️⃣ Hashtags You Could Borrow from the Competitor</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>#️⃣ Hashtags para Robar del Competidor</t>
+          <t>#️⃣ Hashtags que Podrías Tomar del Competidor</t>
         </is>
       </c>
     </row>
@@ -5892,17 +5892,17 @@
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>Rakibin bu videosu {views} izlenmiş. Bu konsept henüz piyasayı kasıp kavurmuyor, ekstra yaratıcılığını konuşturman gerekecek.</t>
+          <t>Rakibin bu videosu {views} izlenmiş. Bu konsept henüz piyasayı kasıp kavurmuyor, ekstra yaratıcılığını konuşturmayı deneyebilirsin.</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>Your competitor's video has {views} views. This concept hasn't dominated the market yet — you'll need extra creativity.</t>
+          <t>Your competitor's video has {views} views. This concept hasn't dominated the market yet — you could bring in some extra creativity.</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>El video de tu competidor tiene {views} vistas. Este concepto aún no ha dominado el mercado — necesitarás creatividad extra.</t>
+          <t>El video de tu competidor tiene {views} vistas. Este concepto aún no ha dominado el mercado — podrías aportar algo de creatividad extra.</t>
         </is>
       </c>
     </row>
@@ -6024,17 +6024,17 @@
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>🥊 AI COACH REÇETESİ</t>
+          <t>🥊 AI KOÇ ÖNERİLERİ</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>🥊 AI COACH PRESCRIPTION</t>
+          <t>🥊 AI COACH SUGGESTIONS</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>🥊 PRESCRIPCIÓN DEL ENTRENADOR IA</t>
+          <t>🥊 SUGERENCIAS DEL ENTRENADOR IA</t>
         </is>
       </c>
     </row>
@@ -6090,17 +6090,17 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Şimdi şunları yap (Acil Eylem Listesi)</t>
+          <t>Bu durumda şunları deneyebilirsin (Öneri Listesi)</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>Do these now (Urgent Action List)</t>
+          <t>In this situation you could try these (Suggestion List)</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>Haz esto ahora (Lista de Acciones Urgentes)</t>
+          <t>En esta situación podrías probar esto (Lista de Sugerencias)</t>
         </is>
       </c>
     </row>
@@ -6178,17 +6178,17 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>KAPAK EMRİ: Şaşırmış/heyecanlı yüz ekle, CTR %40 artar!</t>
+          <t>KAPAK ÖNERİSİ: Şaşırmış/heyecanlı bir yüz eklemeyi deneyebilirsin; bu tıklanma oranını artırmaya yardımcı olabilir.</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>THUMBNAIL ORDER: Add a surprised/excited face, CTR increases by 40%!</t>
+          <t>THUMBNAIL SUGGESTION: You could try adding a surprised/excited face; this may help improve your click-through rate.</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>ORDEN DE MINIATURA: Añade una cara sorprendida/emocionada, ¡el CTR aumenta un 40%!</t>
+          <t>SUGERENCIA DE MINIATURA: Podrías probar a añadir una cara sorprendida/emocionada; esto puede ayudar a mejorar tu tasa de clics.</t>
         </is>
       </c>
     </row>
@@ -6222,17 +6222,17 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>İLK 5-8 SANİYE EMRİ: 'Neden izlesin' cümlesi koy.</t>
+          <t>İLK 5-8 SANİYE ÖNERİSİ: Girişe “neden izlemeli” cümlesi eklemeyi deneyebilirsin.</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>FIRST 5-8 SECONDS ORDER: Add a 'Why should I watch?' sentence.</t>
+          <t>FIRST 5-8 SECONDS SUGGESTION: You could try adding a “why should I watch this?” sentence to your intro.</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>ORDEN DE PRIMEROS 5-8 SEGUNDOS: Añade una frase de '¿Por qué debería verlo?'.</t>
+          <t>SUGERENCIA PARA LOS PRIMEROS 5-8 SEGUNDOS: Podrías probar a añadir una frase de “¿por qué debería verlo?” en la intro.</t>
         </is>
       </c>
     </row>
@@ -6288,17 +6288,17 @@
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>PATLAMA EMRİ: Her 6-8 saniyede cut/zoom/ses efekti ekle.</t>
+          <t>TEMPO ÖNERİSİ: Her 6-8 saniyede bir cut/zoom/ses efekti eklemeyi deneyebilirsin.</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>PEAK ORDER: Add cut/zoom/sound effect every 6-8 seconds.</t>
+          <t>TEMPO SUGGESTION: You could try adding a cut/zoom/sound effect every 6-8 seconds.</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>ORDEN DE PICOS: Añade corte/zoom/efecto de sonido cada 6-8 segundos.</t>
+          <t>SUGERENCIA DE TEMPO: Podrías probar a añadir un corte/zoom/efecto de sonido cada 6-8 segundos.</t>
         </is>
       </c>
     </row>
@@ -6354,17 +6354,17 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>SEO EMRİ: Başlık kelimelerini açıklamanın ilk 200 karakterine ekle.</t>
+          <t>SEO ÖNERİSİ: Başlık kelimelerini açıklamanın ilk 200 karakterine eklemeyi deneyebilirsin.</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>SEO ORDER: Place title keywords in the first 200 characters of description.</t>
+          <t>SEO SUGGESTION: You could try placing your title keywords in the first 200 characters of the description.</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>ORDEN SEO: Coloca palabras clave del título en los primeros 200 caracteres de la descripción.</t>
+          <t>SUGERENCIA SEO: Podrías probar a colocar las palabras clave del título en los primeros 200 caracteres de la descripción.</t>
         </is>
       </c>
     </row>
@@ -6398,17 +6398,17 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>Acil eylem gerekmiyor.</t>
+          <t>Şu an ek bir öneri yok.</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>No urgent action required.</t>
+          <t>No additional suggestions right now.</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>No se requiere acción urgente.</t>
+          <t>No hay sugerencias adicionales por ahora.</t>
         </is>
       </c>
     </row>
@@ -6464,17 +6464,17 @@
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>SEO puanın {seo}/10 ile güçlü — video aramalarda üst sıralarda çıkacak. Ancak Kapak puanın {thumb}/10 ile zayıf. Bu durum videonun aramalarda görünmesine rağmen tıklanmayacağı anlamına gelir. En iyi SEO bile zayıf bir kapakla boşa gider — kapağını acil güncelle!</t>
+          <t>SEO puanın {seo}/10 ile güçlü — video aramalarda üst sıralarda çıkabilir. Ancak Kapak puanın {thumb}/10 ile zayıf. Bu durumda video aramalarda görünse bile tıklanma alması zorlaşabilir. Kapağını güçlendirmeyi düşünebilirsin.</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
-          <t>Your SEO score is strong at {seo}/10 — the video will rank well in searches. However your Thumbnail score is weak at {thumb}/10. This means the video may appear in searches but won't get clicked. Even the best SEO is wasted on a weak thumbnail — update your thumbnail urgently!</t>
+          <t>Your SEO score is strong at {seo}/10 — the video can rank well in searches. However your Thumbnail score is weak at {thumb}/10. In this case the video may appear in searches but still struggle to get clicks. You could consider strengthening your thumbnail.</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr">
         <is>
-          <t>Tu puntuación SEO es fuerte con {seo}/10 — el video aparecerá bien en búsquedas. Sin embargo tu puntuación de Miniatura es débil con {thumb}/10. Esto significa que el video puede aparecer en búsquedas pero no recibirá clics. ¡Incluso el mejor SEO se desperdicia con una miniatura débil — actualiza tu miniatura urgentemente!</t>
+          <t>Tu puntuación SEO es fuerte con {seo}/10 — el video puede posicionarse bien en las búsquedas. Sin embargo, tu puntuación de Miniatura es débil con {thumb}/10. En ese caso el video puede aparecer en búsquedas pero costarle recibir clics. Podrías considerar mejorar tu miniatura.</t>
         </is>
       </c>
     </row>
@@ -6486,17 +6486,17 @@
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>Kapak puanın {thumb}/10 ile çok iyi — izleyici tıklamaya hazır. Ancak SEO puanın {seo}/10 ile düşük, video aramalarda yeterince görünmüyor. Harika bir kapak ama kimse videoyu bulamıyorsa tıklama da olmaz — SEO'nu düzelt!</t>
+          <t>Kapak puanın {thumb}/10 ile çok iyi — izleyici tıklamaya hazır. Ancak SEO puanın {seo}/10 ile düşük, video aramalarda yeterince görünmüyor. Kapak harika olsa da videoyu bulan olmazsa tıklanma zor olabilir; SEO tarafını güçlendirmeyi düşünebilirsin.</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>Your Thumbnail score is excellent at {thumb}/10 — viewers are ready to click. However your SEO score is low at {seo}/10, so the video isn't showing up enough in searches. A great thumbnail is useless if nobody can find the video — fix your SEO!</t>
+          <t>Your Thumbnail score is excellent at {thumb}/10 — viewers are ready to click. However your SEO score is low at {seo}/10, so the video isn't showing up enough in searches. Even a great thumbnail may get few clicks if nobody finds the video; you could consider strengthening your SEO.</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
-          <t>Tu puntuación de Miniatura es excelente con {thumb}/10 — los espectadores están listos para hacer clic. Sin embargo tu puntuación SEO es baja con {seo}/10, por lo que el video no aparece suficientemente en búsquedas. ¡Una gran miniatura es inútil si nadie puede encontrar el video — arregla tu SEO!</t>
+          <t>Tu puntuación de Miniatura es excelente con {thumb}/10 — los espectadores están listos para hacer clic. Sin embargo, tu puntuación SEO es baja con {seo}/10, así que el video no aparece lo suficiente en las búsquedas. Aunque la miniatura sea genial, puede recibir pocos clics si nadie encuentra el video; podrías considerar reforzar tu SEO.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(v6.4.0): complete analysis even when no comparable rival is found
</commit_message>
<xml_diff>
--- a/translations.xlsx
+++ b/translations.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D165"/>
+  <dimension ref="A1:D170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -4079,6 +4079,116 @@
       <c r="D165" s="3" t="inlineStr">
         <is>
           <t>En esta situación podrías probar:</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>compSkipped</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Bu Analizde Rakip Kıyası Yok</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>No Rival Comparison in This Analysis</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Sin Comparación de Rival en Este Análisis</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>compNoMatch</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Bu videoya gerçekten yakın, aynı nişten bir rakip video bulunamadı. Alakasız bir videoyla kıyaslamak yanıltıcı olacağı için bu bölümü boş bıraktık — analizin geri kalanı eksiksiz. Aklında uygun bir video varsa linkini girip yeniden analiz edebilirsin.</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>We could not find a rival video close enough to yours in the same niche. Comparing you with something unrelated would be misleading, so we left this section out — the rest of your analysis is complete. If you have a suitable video in mind, you could paste its link and run the analysis again.</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>No encontramos un video rival lo bastante cercano al tuyo en el mismo nicho. Compararte con algo no relacionado sería engañoso, así que dejamos esta sección fuera; el resto de tu análisis está completo. Si tienes un video adecuado en mente, podrías pegar su enlace y repetir el análisis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>compUrlFailed</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Girdiğin rakip video linki okunamadı, bu yüzden kıyas bölümü atlandı. Analizin geri kalanı eksiksiz. Linki kontrol edip yeniden deneyebilirsin.</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>The rival video link you entered could not be read, so the comparison was skipped. The rest of your analysis is complete. You could check the link and try again.</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>No se pudo leer el enlace del video rival que ingresaste, así que se omitió la comparación. El resto de tu análisis está completo. Podrías revisar el enlace e intentarlo de nuevo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>compLookupFailed</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Rakip araması sırasında YouTube'a ulaşılamadı, bu yüzden kıyas bölümü atlandı. Analizin geri kalanı eksiksiz. Bağlantını kontrol edip yeniden deneyebilirsin.</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>YouTube could not be reached during the rival search, so the comparison was skipped. The rest of your analysis is complete. You could check your connection and try again.</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>No se pudo conectar con YouTube durante la búsqueda del rival, así que se omitió la comparación. El resto de tu análisis está completo. Podrías revisar tu conexión e intentarlo de nuevo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>compViews</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>İzlenme</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>views</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>visualizaciones</t>
         </is>
       </c>
     </row>
@@ -4093,7 +4203,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D124"/>
+  <dimension ref="A1:D125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -6830,6 +6940,28 @@
         </is>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>no_competitor_desc</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Bu videoya yakın, aynı nişten kıyaslanabilir bir rakip video bulunamadı. Alakasız bir videoyla kıyaslamak yanıltıcı olacağı için bu bölüm boş bırakıldı. Raporun geri kalanı eksiksizdir; uygun bir rakip videonun linkini girerek yeniden analiz edebilirsin.</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>No rival video close enough to yours in the same niche was found. Comparing against something unrelated would be misleading, so this section was left out. The rest of the report is complete; you could paste the link of a suitable rival video and run the analysis again.</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>No se encontró un video rival lo bastante cercano al tuyo en el mismo nicho. Comparar con algo no relacionado sería engañoso, por eso se omitió esta sección. El resto del informe está completo; podrías pegar el enlace de un video rival adecuado y repetir el análisis.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>